<commit_message>
chore(lab-5): add new tree model results
</commit_message>
<xml_diff>
--- a/lab_5/models/metrics/catboost.xlsx
+++ b/lab_5/models/metrics/catboost.xlsx
@@ -467,163 +467,163 @@
     </row>
     <row r="2">
       <c r="A2" t="n">
-        <v>0.9415</v>
+        <v>0.9408</v>
       </c>
       <c r="B2" t="n">
-        <v>0.8238</v>
+        <v>0.8575</v>
       </c>
       <c r="C2" t="n">
-        <v>0.053</v>
+        <v>0.09520000000000001</v>
       </c>
       <c r="D2" t="n">
-        <v>0.8889</v>
+        <v>0.5881999999999999</v>
       </c>
       <c r="E2" t="n">
-        <v>0.1</v>
+        <v>0.1639</v>
       </c>
       <c r="F2" t="n">
-        <v>0.09370000000000001</v>
+        <v>0.1495</v>
       </c>
       <c r="G2" t="n">
-        <v>0.2089</v>
+        <v>0.22</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="n">
-        <v>0.9403</v>
+        <v>0.9385</v>
       </c>
       <c r="B3" t="n">
-        <v>0.8334</v>
+        <v>0.8361</v>
       </c>
       <c r="C3" t="n">
-        <v>0.04</v>
+        <v>0.09429999999999999</v>
       </c>
       <c r="D3" t="n">
-        <v>0.6667</v>
+        <v>0.5</v>
       </c>
       <c r="E3" t="n">
-        <v>0.0755</v>
+        <v>0.1587</v>
       </c>
       <c r="F3" t="n">
-        <v>0.06909999999999999</v>
+        <v>0.142</v>
       </c>
       <c r="G3" t="n">
-        <v>0.1534</v>
+        <v>0.1978</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="n">
-        <v>0.9411</v>
+        <v>0.9414</v>
       </c>
       <c r="B4" t="n">
-        <v>0.8418</v>
+        <v>0.8453000000000001</v>
       </c>
       <c r="C4" t="n">
-        <v>0.0667</v>
+        <v>0.0857</v>
       </c>
       <c r="D4" t="n">
-        <v>0.6667</v>
+        <v>0.6429</v>
       </c>
       <c r="E4" t="n">
-        <v>0.1212</v>
+        <v>0.1513</v>
       </c>
       <c r="F4" t="n">
-        <v>0.1114</v>
+        <v>0.1389</v>
       </c>
       <c r="G4" t="n">
-        <v>0.1983</v>
+        <v>0.2202</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="n">
-        <v>0.9415</v>
+        <v>0.9414</v>
       </c>
       <c r="B5" t="n">
-        <v>0.847</v>
+        <v>0.8003</v>
       </c>
       <c r="C5" t="n">
-        <v>0.0533</v>
+        <v>0.0571</v>
       </c>
       <c r="D5" t="n">
-        <v>0.8</v>
+        <v>0.75</v>
       </c>
       <c r="E5" t="n">
-        <v>0.1</v>
+        <v>0.1062</v>
       </c>
       <c r="F5" t="n">
-        <v>0.0931</v>
+        <v>0.0984</v>
       </c>
       <c r="G5" t="n">
-        <v>0.1973</v>
+        <v>0.1967</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="n">
-        <v>0.9399</v>
+        <v>0.9414</v>
       </c>
       <c r="B6" t="n">
-        <v>0.8356</v>
+        <v>0.8491</v>
       </c>
       <c r="C6" t="n">
-        <v>0.0331</v>
+        <v>0.0571</v>
       </c>
       <c r="D6" t="n">
-        <v>0.7143</v>
+        <v>0.75</v>
       </c>
       <c r="E6" t="n">
-        <v>0.0633</v>
+        <v>0.1062</v>
       </c>
       <c r="F6" t="n">
-        <v>0.0582</v>
+        <v>0.0984</v>
       </c>
       <c r="G6" t="n">
-        <v>0.1453</v>
+        <v>0.1967</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="n">
-        <v>0.9409</v>
+        <v>0.9407</v>
       </c>
       <c r="B7" t="n">
-        <v>0.8363</v>
+        <v>0.8377</v>
       </c>
       <c r="C7" t="n">
-        <v>0.0492</v>
+        <v>0.0779</v>
       </c>
       <c r="D7" t="n">
-        <v>0.7473</v>
+        <v>0.6462</v>
       </c>
       <c r="E7" t="n">
-        <v>0.092</v>
+        <v>0.1373</v>
       </c>
       <c r="F7" t="n">
-        <v>0.0851</v>
+        <v>0.1254</v>
       </c>
       <c r="G7" t="n">
-        <v>0.1806</v>
+        <v>0.2063</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="n">
-        <v>0.0007</v>
+        <v>0.0011</v>
       </c>
       <c r="B8" t="n">
-        <v>0.007900000000000001</v>
+        <v>0.0199</v>
       </c>
       <c r="C8" t="n">
-        <v>0.0117</v>
+        <v>0.0173</v>
       </c>
       <c r="D8" t="n">
-        <v>0.0859</v>
+        <v>0.09619999999999999</v>
       </c>
       <c r="E8" t="n">
-        <v>0.0204</v>
+        <v>0.0257</v>
       </c>
       <c r="F8" t="n">
-        <v>0.019</v>
+        <v>0.0223</v>
       </c>
       <c r="G8" t="n">
-        <v>0.026</v>
+        <v>0.0113</v>
       </c>
     </row>
   </sheetData>

</xml_diff>